<commit_message>
Deep SEO audit fixes: canonical order variants, plans Product schema, heading outline, content depth, city differentiation, meta lengths, caching
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AbMcYcKjt6GmZtWm6wMckD
</commit_message>
<xml_diff>
--- a/docs/keyword-map.xlsx
+++ b/docs/keyword-map.xlsx
@@ -440,7 +440,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>/root/.claude/uploads/5a4562d9-198c-51ab-b817-8b92809dcb72/d56f9b2b-Keyword_Canada.xlsx</t>
+          <t>/root/.claude/uploads/5a4562d9-198c-51ab-b817-8b92809dcb72/7d244209-Keyword_Canada.xlsx</t>
         </is>
       </c>
     </row>
@@ -36708,7 +36708,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Formuler Z11 Pro Max &amp; Z-Series IPTV Box Guide (2026) | IPTVMaple</t>
+          <t>Formuler Z-Series IPTV Box Guide (2026) | IPTVMaple</t>
         </is>
       </c>
     </row>
@@ -38266,7 +38266,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Best IPTV for Sports in Canada (2026): NHL, UFC, NBA | IPTVMaple</t>
+          <t>Best IPTV for Sports in Canada (2026): NHL, UFC | IPTVMaple</t>
         </is>
       </c>
     </row>

</xml_diff>